<commit_message>
Actualizacion y despliegue controller comercial: 25/09/2026
</commit_message>
<xml_diff>
--- a/Pedidos 25.09 comerciales.xlsx
+++ b/Pedidos 25.09 comerciales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agroquimicacodiagro365-my.sharepoint.com/personal/oscar_ocampo_codiagro_com/Documents/Escritorio/Presupuesto 2026/Calsif Comerciales/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B6F85475-2B33-4F32-A2B6-2A82AD562D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{B6F85475-2B33-4F32-A2B6-2A82AD562D5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{474AC842-0D6D-4404-812B-9417AAB7C36B}"/>
   <bookViews>
     <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{847F4FF8-4678-4360-B38A-3C989DB4B87F}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="LineasPedidoCliente (2)" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="DatosExternos_1" localSheetId="0" hidden="1">'LineasPedidoCliente (2)'!$A$1:$P$178</definedName>
     <definedName name="DatosExternos_1" localSheetId="0" hidden="1">'LineasPedidoCliente (2)'!$A$1:$P$178</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -1028,7 +1027,45 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{EAB99023-CBC2-4CDC-95F8-CAF9867A69DF}" name="LineasPedidoCliente4" displayName="LineasPedidoCliente4" ref="A1:P178" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:P178" xr:uid="{6292CA43-A9C0-4280-B40A-9DD133760E8A}"/>
+  <autoFilter ref="A1:P178" xr:uid="{6292CA43-A9C0-4280-B40A-9DD133760E8A}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="ACTIV. PRODUC. Y COMERC. LA VEGUILLA, SL"/>
+        <filter val="AGRONEW FITO, S.L."/>
+        <filter val="AGROQUIMICAS DRAGO S.L."/>
+        <filter val="AGROTÉCNICA DEL NORTE, S.L"/>
+        <filter val="AGROVEYCA,S.L"/>
+        <filter val="AIFAR S.P.A"/>
+        <filter val="ALMENDRALIA IBÉRICA, S.L.U."/>
+        <filter val="ASESORAMIENTO TECNICO DE CULTIVOS, S.L."/>
+        <filter val="ASOC. HORTICULTORES DE VILLA DEL PRADO"/>
+        <filter val="BARDENAS COMERCIAL, S.L."/>
+        <filter val="CABRERA MORALES FRANCISCO"/>
+        <filter val="CAMPOEJIDO S.C.A."/>
+        <filter val="ÇITAR ÇIÇEK TARIM TIC. LTD. STI"/>
+        <filter val="CODIMED EXPORT, S.L."/>
+        <filter val="COMERCIAL NORTE AGROCAMPO, S.L."/>
+        <filter val="COMERCIAL TÉCNICA FITOCARTHAGO, S.L."/>
+        <filter val="DOTRA CHEMICALS"/>
+        <filter val="DOTRA GULF TRADING COMPANY"/>
+        <filter val="ECUAQUIMICA"/>
+        <filter val="EUROFERTIL, S.A."/>
+        <filter val="FINCA DOÑA ANA C.B."/>
+        <filter val="FITOMURCIA S.L."/>
+        <filter val="FITOSANITARIOS CARCAIXENT, S.L."/>
+        <filter val="FITOSANITARIOS DRAGO S.L.U"/>
+        <filter val="FITOXENT S.C.L.V."/>
+        <filter val="GUIVARTO AGRICOLA, S.L."/>
+        <filter val="MAJ AGROQUIMICOS S.L."/>
+        <filter val="SAFIAGRO, S.A."/>
+        <filter val="SC MARCOSER S.R.L."/>
+        <filter val="SERVIAGRI´ 97, S.L."/>
+        <filter val="SUCA, S.C.A."/>
+        <filter val="T.J AGRICULTURA S.L."/>
+        <filter val="VILLALTA SATIVUM, S.L."/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P178">
     <sortCondition ref="A1:A178"/>
   </sortState>
@@ -3092,7 +3129,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1">
         <v>46268</v>
       </c>
@@ -3142,7 +3179,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1">
         <v>46268</v>
       </c>
@@ -3192,7 +3229,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1">
         <v>46268</v>
       </c>
@@ -3242,7 +3279,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1">
         <v>46268</v>
       </c>
@@ -3292,7 +3329,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1">
         <v>46268</v>
       </c>
@@ -3342,7 +3379,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1">
         <v>46268</v>
       </c>
@@ -3392,7 +3429,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1">
         <v>46268</v>
       </c>
@@ -3442,7 +3479,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1">
         <v>46268</v>
       </c>
@@ -3492,7 +3529,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="1">
         <v>46268</v>
       </c>
@@ -3542,7 +3579,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1">
         <v>46268</v>
       </c>
@@ -3592,7 +3629,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="1">
         <v>46268</v>
       </c>
@@ -3642,7 +3679,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="1">
         <v>46268</v>
       </c>
@@ -3692,7 +3729,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1">
         <v>46268</v>
       </c>
@@ -3742,7 +3779,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="1">
         <v>46268</v>
       </c>
@@ -3792,7 +3829,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="1">
         <v>46268</v>
       </c>
@@ -3842,7 +3879,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="1">
         <v>46268</v>
       </c>
@@ -3892,7 +3929,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="1">
         <v>46268</v>
       </c>
@@ -9792,7 +9829,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="169" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:16" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" s="1">
         <v>46288</v>
       </c>

</xml_diff>